<commit_message>
Updated example dataset reports.
</commit_message>
<xml_diff>
--- a/example/reference_results/5_dada2_pipeline/processing_summary.xlsx
+++ b/example/reference_results/5_dada2_pipeline/processing_summary.xlsx
@@ -7,7 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Reads_Tracking" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Column_Dictionary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Database_Comparison" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Column_Dictionary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -154,8 +155,78 @@
 </comments>
 </file>
 
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author/>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Taxonomic rank being evaluated for classification success: Kingdom, Phylum, Class, Order, Family, Genus, or Species.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Number of ASVs assigned a non-missing, non-empty taxonomic label at this rank using the SILVA reference database.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Number of ASVs assigned a non-missing, non-empty taxonomic label at this rank using the GTDB reference database.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Percentage of all ASVs classified at this rank by SILVA, calculated as SILVA_Classified / total ASVs * 100.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <name val="Tahoma"/>
+          </rPr>
+          <t xml:space="preserve">Percentage of all ASVs classified at this rank by GTDB, calculated as GTDB_Classified / total ASVs * 100.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="64">
   <si>
     <t xml:space="preserve">SampleID</t>
   </si>
@@ -250,6 +321,42 @@
     <t xml:space="preserve">Mouse-F3-Day-150</t>
   </si>
   <si>
+    <t xml:space="preserve">Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SILVA_Classified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTDB_Classified</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SILVA_Percent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GTDB_Percent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kingdom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phylum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Class</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Species</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sheet</t>
   </si>
   <si>
@@ -293,6 +400,24 @@
   </si>
   <si>
     <t xml:space="preserve">Percentage of this sample's raw input reads that survived the entire pipeline through chimera removal, calculated as Non_Chimeric / Raw_Reads * 100.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Database_Comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taxonomic rank being evaluated for classification success: Kingdom, Phylum, Class, Order, Family, Genus, or Species.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of ASVs assigned a non-missing, non-empty taxonomic label at this rank using the SILVA reference database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of ASVs assigned a non-missing, non-empty taxonomic label at this rank using the GTDB reference database.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentage of all ASVs classified at this rank by SILVA, calculated as SILVA_Classified / total ASVs * 100.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percentage of all ASVs classified at this rank by GTDB, calculated as GTDB_Classified / total ASVs * 100.</t>
   </si>
 </sst>
 </file>
@@ -369,8 +494,22 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:C12" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:C12"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:E8" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:E8"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Level"/>
+    <tableColumn id="2" name="SILVA_Classified"/>
+    <tableColumn id="3" name="GTDB_Classified"/>
+    <tableColumn id="4" name="SILVA_Percent"/>
+    <tableColumn id="5" name="GTDB_Percent"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:C17" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:C17"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Sheet"/>
     <tableColumn id="2" name="Column"/>
@@ -1431,148 +1570,364 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="14.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="7.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="13.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="n">
+        <v>232</v>
+      </c>
+      <c r="C2" t="n">
+        <v>232</v>
+      </c>
+      <c r="D2" t="n">
+        <v>100</v>
+      </c>
+      <c r="E2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="n">
+        <v>232</v>
+      </c>
+      <c r="C3" t="n">
+        <v>228</v>
+      </c>
+      <c r="D3" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" t="n">
+        <v>98.3</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" t="n">
+        <v>232</v>
+      </c>
+      <c r="C4" t="n">
+        <v>228</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E4" t="n">
+        <v>98.3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B5" t="n">
+        <v>231</v>
+      </c>
+      <c r="C5" t="n">
+        <v>223</v>
+      </c>
+      <c r="D5" t="n">
+        <v>99.6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>96.1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="n">
+        <v>209</v>
+      </c>
+      <c r="C6" t="n">
+        <v>220</v>
+      </c>
+      <c r="D6" t="n">
+        <v>90.1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>94.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="n">
+        <v>107</v>
+      </c>
+      <c r="C7" t="n">
+        <v>103</v>
+      </c>
+      <c r="D7" t="n">
+        <v>46.1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>44.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" t="n">
+        <v>29</v>
+      </c>
+      <c r="C8" t="n">
+        <v>53</v>
+      </c>
+      <c r="D8" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="E8" t="n">
+        <v>22.8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <legacyDrawing r:id="rIdvml"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <sheetPr>
+    <tabColor rgb="FFAF7AA1"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="19.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="28.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="250.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B3" t="s">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
         <v>3</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
         <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B11" t="s">
         <v>9</v>
       </c>
       <c r="C11" t="s">
-        <v>44</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
         <v>10</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>